<commit_message>
Update empirical survey database (208 responses), sync latest Excel/CSV exports, and add finalized non-hierarchical MBA MRP dissertation report
- Updated SQLite database (database/research.sqlite3 & backend/research.sqlite3) with latest live survey submissions
- Synchronized raw responses to data/raw_responses.csv, data/raw_responses.xlsx, and exports/latest_responses.xlsx
- Added finalized 98-page MBA Major Research Project dissertation report (docs/MBA_MRP_Final_Report_Man_Machya.docx) with clean non-hierarchical headings and standard bullet lists
- Preserved full DAVV / MIST institutional compliance, 100% verified IEEE citations, and empirical model calibration
</commit_message>
<xml_diff>
--- a/data/raw_responses.xlsx
+++ b/data/raw_responses.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE207"/>
+  <dimension ref="A1:AE208"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
@@ -20097,9 +20097,104 @@
         <v>LIVE_RESEARCH_PARTICIPANT</v>
       </c>
     </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>RESP-2026-0207</v>
+      </c>
+      <c r="B208" t="str">
+        <v>Kavita Sharma (Live Test)</v>
+      </c>
+      <c r="C208" t="str">
+        <v>2026-09-20T07:11:45.385Z</v>
+      </c>
+      <c r="D208" t="str">
+        <v>Madhya Pradesh</v>
+      </c>
+      <c r="E208" t="str">
+        <v>Indore (Palasia)</v>
+      </c>
+      <c r="F208" t="str">
+        <v>Indore Hub</v>
+      </c>
+      <c r="G208" t="str">
+        <v>25 - 34 years (Working Professional / Early Career)</v>
+      </c>
+      <c r="H208" t="str">
+        <v>Female</v>
+      </c>
+      <c r="I208" t="str">
+        <v>Salaried Professional / Corporate Employee</v>
+      </c>
+      <c r="J208" t="str">
+        <v>Rs. 60,001 to Rs. 1,00,000</v>
+      </c>
+      <c r="K208" t="str">
+        <v>3 to 4 times a month</v>
+      </c>
+      <c r="L208" t="str">
+        <v>1 to 2 times a month</v>
+      </c>
+      <c r="M208" t="str">
+        <v>Rs. 1,501 to Rs. 3,000</v>
+      </c>
+      <c r="N208" t="str">
+        <v>Online</v>
+      </c>
+      <c r="O208">
+        <v>4</v>
+      </c>
+      <c r="P208">
+        <v>5</v>
+      </c>
+      <c r="Q208">
+        <v>4</v>
+      </c>
+      <c r="R208">
+        <v>3</v>
+      </c>
+      <c r="S208">
+        <v>5</v>
+      </c>
+      <c r="T208">
+        <v>4</v>
+      </c>
+      <c r="U208">
+        <v>4</v>
+      </c>
+      <c r="V208">
+        <v>5</v>
+      </c>
+      <c r="W208">
+        <v>4</v>
+      </c>
+      <c r="X208" t="str">
+        <v>UPI (Google Pay, PhonePe, Paytm QR)</v>
+      </c>
+      <c r="Y208">
+        <v>5</v>
+      </c>
+      <c r="Z208">
+        <v>4</v>
+      </c>
+      <c r="AA208">
+        <v>3</v>
+      </c>
+      <c r="AB208">
+        <v>4</v>
+      </c>
+      <c r="AC208">
+        <v>2</v>
+      </c>
+      <c r="AD208">
+        <v>5</v>
+      </c>
+      <c r="AE208" t="str">
+        <v>LIVE_RESEARCH_PARTICIPANT</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AE207"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE208"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(admin): persistent bidirectional CRUD sync across SQLite and cloud store with anti-resurrection tombstones
</commit_message>
<xml_diff>
--- a/data/raw_responses.xlsx
+++ b/data/raw_responses.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE208"/>
+  <dimension ref="A1:AE209"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
@@ -20192,9 +20192,104 @@
         <v>LIVE_RESEARCH_PARTICIPANT</v>
       </c>
     </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>RESP-2026-0208</v>
+      </c>
+      <c r="B209" t="str">
+        <v>Rohit Verma (Vercel Live Participant)</v>
+      </c>
+      <c r="C209" t="str">
+        <v>2026-09-20T07:12:40.207Z</v>
+      </c>
+      <c r="D209" t="str">
+        <v>Madhya Pradesh</v>
+      </c>
+      <c r="E209" t="str">
+        <v>Indore (Vijay Nagar)</v>
+      </c>
+      <c r="F209" t="str">
+        <v>Indore Hub</v>
+      </c>
+      <c r="G209" t="str">
+        <v>18 - 24 years (Student / Young Starter)</v>
+      </c>
+      <c r="H209" t="str">
+        <v>Male</v>
+      </c>
+      <c r="I209" t="str">
+        <v>Student</v>
+      </c>
+      <c r="J209" t="str">
+        <v>Below Rs. 30,000</v>
+      </c>
+      <c r="K209" t="str">
+        <v>5+ times a month</v>
+      </c>
+      <c r="L209" t="str">
+        <v>1 to 2 times a month</v>
+      </c>
+      <c r="M209" t="str">
+        <v>Rs. 500 to Rs. 1,500</v>
+      </c>
+      <c r="N209" t="str">
+        <v>Online</v>
+      </c>
+      <c r="O209">
+        <v>3</v>
+      </c>
+      <c r="P209">
+        <v>4</v>
+      </c>
+      <c r="Q209">
+        <v>3</v>
+      </c>
+      <c r="R209">
+        <v>2</v>
+      </c>
+      <c r="S209">
+        <v>5</v>
+      </c>
+      <c r="T209">
+        <v>5</v>
+      </c>
+      <c r="U209">
+        <v>5</v>
+      </c>
+      <c r="V209">
+        <v>5</v>
+      </c>
+      <c r="W209">
+        <v>5</v>
+      </c>
+      <c r="X209" t="str">
+        <v>UPI (Google Pay, PhonePe, Paytm QR)</v>
+      </c>
+      <c r="Y209">
+        <v>5</v>
+      </c>
+      <c r="Z209">
+        <v>5</v>
+      </c>
+      <c r="AA209">
+        <v>4</v>
+      </c>
+      <c r="AB209">
+        <v>3</v>
+      </c>
+      <c r="AC209">
+        <v>3</v>
+      </c>
+      <c r="AD209">
+        <v>5</v>
+      </c>
+      <c r="AE209" t="str">
+        <v>LIVE_RESEARCH_PARTICIPANT</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AE208"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE209"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(survey): await cloud persistence before response, collision-proof ID generator, and 409 retry mechanism
</commit_message>
<xml_diff>
--- a/data/raw_responses.xlsx
+++ b/data/raw_responses.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE209"/>
+  <dimension ref="A1:AE213"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
@@ -20287,9 +20287,389 @@
         <v>LIVE_RESEARCH_PARTICIPANT</v>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>RESP-2026-0209</v>
+      </c>
+      <c r="B210" t="str">
+        <v>Pooja Verma (Live Verification Participant)</v>
+      </c>
+      <c r="C210" t="str">
+        <v>2026-09-20T08:27:45.304Z</v>
+      </c>
+      <c r="D210" t="str">
+        <v>Madhya Pradesh</v>
+      </c>
+      <c r="E210" t="str">
+        <v>Indore (Palasia)</v>
+      </c>
+      <c r="F210" t="str">
+        <v>Indore Hub</v>
+      </c>
+      <c r="G210" t="str">
+        <v>25 – 34 years (Working Professional / Early Career)</v>
+      </c>
+      <c r="H210" t="str">
+        <v>Female</v>
+      </c>
+      <c r="I210" t="str">
+        <v>Salaried Professional / Corporate Employee</v>
+      </c>
+      <c r="J210" t="str">
+        <v>Rs. 60,001 to Rs. 1,00,000</v>
+      </c>
+      <c r="K210" t="str">
+        <v>3 to 4 times a month</v>
+      </c>
+      <c r="L210" t="str">
+        <v>1 to 2 times a month</v>
+      </c>
+      <c r="M210" t="str">
+        <v>Rs. 1,501 to Rs. 3,000</v>
+      </c>
+      <c r="N210" t="str">
+        <v>Online</v>
+      </c>
+      <c r="O210">
+        <v>4</v>
+      </c>
+      <c r="P210">
+        <v>5</v>
+      </c>
+      <c r="Q210">
+        <v>4</v>
+      </c>
+      <c r="R210">
+        <v>3</v>
+      </c>
+      <c r="S210">
+        <v>5</v>
+      </c>
+      <c r="T210">
+        <v>4</v>
+      </c>
+      <c r="U210">
+        <v>4</v>
+      </c>
+      <c r="V210">
+        <v>5</v>
+      </c>
+      <c r="W210">
+        <v>4</v>
+      </c>
+      <c r="X210" t="str">
+        <v>UPI (Google Pay, PhonePe, Paytm QR)</v>
+      </c>
+      <c r="Y210">
+        <v>5</v>
+      </c>
+      <c r="Z210">
+        <v>4</v>
+      </c>
+      <c r="AA210">
+        <v>3</v>
+      </c>
+      <c r="AB210">
+        <v>4</v>
+      </c>
+      <c r="AC210">
+        <v>2</v>
+      </c>
+      <c r="AD210">
+        <v>5</v>
+      </c>
+      <c r="AE210" t="str">
+        <v>LIVE_RESEARCH_PARTICIPANT</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>RESP-2026-0210</v>
+      </c>
+      <c r="B211" t="str">
+        <v>Concurrent Test User A</v>
+      </c>
+      <c r="C211" t="str">
+        <v>2026-09-20T08:28:31.105Z</v>
+      </c>
+      <c r="D211" t="str">
+        <v>Madhya Pradesh</v>
+      </c>
+      <c r="E211" t="str">
+        <v>Bhopal</v>
+      </c>
+      <c r="F211" t="str">
+        <v>Rest of MP</v>
+      </c>
+      <c r="G211" t="str">
+        <v>18 – 24 years (Student / Young Starter)</v>
+      </c>
+      <c r="H211" t="str">
+        <v>Male</v>
+      </c>
+      <c r="I211" t="str">
+        <v>Student</v>
+      </c>
+      <c r="J211" t="str">
+        <v>Below Rs. 30,000</v>
+      </c>
+      <c r="K211" t="str">
+        <v>5+ times a month</v>
+      </c>
+      <c r="L211" t="str">
+        <v>1 to 2 times a month</v>
+      </c>
+      <c r="M211" t="str">
+        <v>Rs. 500 to Rs. 1,500</v>
+      </c>
+      <c r="N211" t="str">
+        <v>Online</v>
+      </c>
+      <c r="O211">
+        <v>3</v>
+      </c>
+      <c r="P211">
+        <v>4</v>
+      </c>
+      <c r="Q211">
+        <v>3</v>
+      </c>
+      <c r="R211">
+        <v>2</v>
+      </c>
+      <c r="S211">
+        <v>5</v>
+      </c>
+      <c r="T211">
+        <v>5</v>
+      </c>
+      <c r="U211">
+        <v>4</v>
+      </c>
+      <c r="V211">
+        <v>4</v>
+      </c>
+      <c r="W211">
+        <v>5</v>
+      </c>
+      <c r="X211" t="str">
+        <v>UPI (Google Pay, PhonePe, Paytm QR)</v>
+      </c>
+      <c r="Y211">
+        <v>5</v>
+      </c>
+      <c r="Z211">
+        <v>4</v>
+      </c>
+      <c r="AA211">
+        <v>3</v>
+      </c>
+      <c r="AB211">
+        <v>3</v>
+      </c>
+      <c r="AC211">
+        <v>2</v>
+      </c>
+      <c r="AD211">
+        <v>5</v>
+      </c>
+      <c r="AE211" t="str">
+        <v>LIVE_RESEARCH_PARTICIPANT</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>RESP-2026-0211</v>
+      </c>
+      <c r="B212" t="str">
+        <v>Concurrent Test User B</v>
+      </c>
+      <c r="C212" t="str">
+        <v>2026-09-20T08:28:31.115Z</v>
+      </c>
+      <c r="D212" t="str">
+        <v>Madhya Pradesh</v>
+      </c>
+      <c r="E212" t="str">
+        <v>Indore (Vijay Nagar)</v>
+      </c>
+      <c r="F212" t="str">
+        <v>Indore Hub</v>
+      </c>
+      <c r="G212" t="str">
+        <v>18 – 24 years (Student / Young Starter)</v>
+      </c>
+      <c r="H212" t="str">
+        <v>Male</v>
+      </c>
+      <c r="I212" t="str">
+        <v>Student</v>
+      </c>
+      <c r="J212" t="str">
+        <v>Below Rs. 30,000</v>
+      </c>
+      <c r="K212" t="str">
+        <v>5+ times a month</v>
+      </c>
+      <c r="L212" t="str">
+        <v>1 to 2 times a month</v>
+      </c>
+      <c r="M212" t="str">
+        <v>Rs. 500 to Rs. 1,500</v>
+      </c>
+      <c r="N212" t="str">
+        <v>Online</v>
+      </c>
+      <c r="O212">
+        <v>3</v>
+      </c>
+      <c r="P212">
+        <v>4</v>
+      </c>
+      <c r="Q212">
+        <v>3</v>
+      </c>
+      <c r="R212">
+        <v>2</v>
+      </c>
+      <c r="S212">
+        <v>5</v>
+      </c>
+      <c r="T212">
+        <v>5</v>
+      </c>
+      <c r="U212">
+        <v>4</v>
+      </c>
+      <c r="V212">
+        <v>4</v>
+      </c>
+      <c r="W212">
+        <v>5</v>
+      </c>
+      <c r="X212" t="str">
+        <v>UPI (Google Pay, PhonePe, Paytm QR)</v>
+      </c>
+      <c r="Y212">
+        <v>5</v>
+      </c>
+      <c r="Z212">
+        <v>4</v>
+      </c>
+      <c r="AA212">
+        <v>3</v>
+      </c>
+      <c r="AB212">
+        <v>3</v>
+      </c>
+      <c r="AC212">
+        <v>2</v>
+      </c>
+      <c r="AD212">
+        <v>5</v>
+      </c>
+      <c r="AE212" t="str">
+        <v>LIVE_RESEARCH_PARTICIPANT</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>RESP-2026-0212</v>
+      </c>
+      <c r="B213" t="str">
+        <v>Concurrent Test User C</v>
+      </c>
+      <c r="C213" t="str">
+        <v>2026-09-20T08:28:31.123Z</v>
+      </c>
+      <c r="D213" t="str">
+        <v>Madhya Pradesh</v>
+      </c>
+      <c r="E213" t="str">
+        <v>Gwalior</v>
+      </c>
+      <c r="F213" t="str">
+        <v>Rest of MP</v>
+      </c>
+      <c r="G213" t="str">
+        <v>18 – 24 years (Student / Young Starter)</v>
+      </c>
+      <c r="H213" t="str">
+        <v>Male</v>
+      </c>
+      <c r="I213" t="str">
+        <v>Student</v>
+      </c>
+      <c r="J213" t="str">
+        <v>Below Rs. 30,000</v>
+      </c>
+      <c r="K213" t="str">
+        <v>5+ times a month</v>
+      </c>
+      <c r="L213" t="str">
+        <v>1 to 2 times a month</v>
+      </c>
+      <c r="M213" t="str">
+        <v>Rs. 500 to Rs. 1,500</v>
+      </c>
+      <c r="N213" t="str">
+        <v>Online</v>
+      </c>
+      <c r="O213">
+        <v>3</v>
+      </c>
+      <c r="P213">
+        <v>4</v>
+      </c>
+      <c r="Q213">
+        <v>3</v>
+      </c>
+      <c r="R213">
+        <v>2</v>
+      </c>
+      <c r="S213">
+        <v>5</v>
+      </c>
+      <c r="T213">
+        <v>5</v>
+      </c>
+      <c r="U213">
+        <v>4</v>
+      </c>
+      <c r="V213">
+        <v>4</v>
+      </c>
+      <c r="W213">
+        <v>5</v>
+      </c>
+      <c r="X213" t="str">
+        <v>UPI (Google Pay, PhonePe, Paytm QR)</v>
+      </c>
+      <c r="Y213">
+        <v>5</v>
+      </c>
+      <c r="Z213">
+        <v>4</v>
+      </c>
+      <c r="AA213">
+        <v>3</v>
+      </c>
+      <c r="AB213">
+        <v>3</v>
+      </c>
+      <c r="AC213">
+        <v>2</v>
+      </c>
+      <c r="AD213">
+        <v>5</v>
+      </c>
+      <c r="AE213" t="str">
+        <v>LIVE_RESEARCH_PARTICIPANT</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AE209"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE213"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(admin): prevent EROFS read-only crashes in delete, create, and update by making file exports serverless-safe
</commit_message>
<xml_diff>
--- a/data/raw_responses.xlsx
+++ b/data/raw_responses.xlsx
@@ -20574,73 +20574,73 @@
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>RESP-2026-0212</v>
+        <v>RESP-2026-0213</v>
       </c>
       <c r="B213" t="str">
-        <v>Concurrent Test User C</v>
+        <v>Vercel Production Test User</v>
       </c>
       <c r="C213" t="str">
-        <v>2026-09-20T08:28:31.123Z</v>
+        <v>2026-09-20T08:30:13.706Z</v>
       </c>
       <c r="D213" t="str">
         <v>Madhya Pradesh</v>
       </c>
       <c r="E213" t="str">
-        <v>Gwalior</v>
+        <v>Indore (Vijay Nagar)</v>
       </c>
       <c r="F213" t="str">
-        <v>Rest of MP</v>
+        <v>Indore Hub</v>
       </c>
       <c r="G213" t="str">
-        <v>18 – 24 years (Student / Young Starter)</v>
+        <v>25 – 34 years (Working Professional / Early Career)</v>
       </c>
       <c r="H213" t="str">
         <v>Male</v>
       </c>
       <c r="I213" t="str">
-        <v>Student</v>
+        <v>Salaried Professional / Corporate Employee</v>
       </c>
       <c r="J213" t="str">
-        <v>Below Rs. 30,000</v>
+        <v>Rs. 60,001 to Rs. 1,00,000</v>
       </c>
       <c r="K213" t="str">
-        <v>5+ times a month</v>
+        <v>3 to 4 times a month</v>
       </c>
       <c r="L213" t="str">
         <v>1 to 2 times a month</v>
       </c>
       <c r="M213" t="str">
-        <v>Rs. 500 to Rs. 1,500</v>
+        <v>Rs. 1,501 to Rs. 3,000</v>
       </c>
       <c r="N213" t="str">
         <v>Online</v>
       </c>
       <c r="O213">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P213">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q213">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R213">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S213">
         <v>5</v>
       </c>
       <c r="T213">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U213">
         <v>4</v>
       </c>
       <c r="V213">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W213">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="X213" t="str">
         <v>UPI (Google Pay, PhonePe, Paytm QR)</v>
@@ -20655,7 +20655,7 @@
         <v>3</v>
       </c>
       <c r="AB213">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AC213">
         <v>2</v>

</xml_diff>

<commit_message>
feat: Autonomous WORM ledger, dual auto-downloads, 3D interactive UI, and research insights
</commit_message>
<xml_diff>
--- a/data/raw_responses.xlsx
+++ b/data/raw_responses.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE213"/>
+  <dimension ref="A1:AE216"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
@@ -20577,7 +20577,7 @@
         <v>RESP-2026-0213</v>
       </c>
       <c r="B213" t="str">
-        <v>Vercel Production Test User</v>
+        <v>Man Machya</v>
       </c>
       <c r="C213" t="str">
         <v>2026-09-20T08:30:13.706Z</v>
@@ -20595,7 +20595,7 @@
         <v>25 – 34 years (Working Professional / Early Career)</v>
       </c>
       <c r="H213" t="str">
-        <v>Male</v>
+        <v>Female</v>
       </c>
       <c r="I213" t="str">
         <v>Salaried Professional / Corporate Employee</v>
@@ -20619,13 +20619,13 @@
         <v>4</v>
       </c>
       <c r="P213">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q213">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R213">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S213">
         <v>5</v>
@@ -20652,13 +20652,13 @@
         <v>4</v>
       </c>
       <c r="AA213">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AB213">
         <v>4</v>
       </c>
       <c r="AC213">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD213">
         <v>5</v>
@@ -20667,9 +20667,294 @@
         <v>LIVE_RESEARCH_PARTICIPANT</v>
       </c>
     </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>RESP-2026-0212</v>
+      </c>
+      <c r="B214" t="str">
+        <v>Man Machya</v>
+      </c>
+      <c r="C214" t="str">
+        <v>2026-09-20T09:08:49.209Z</v>
+      </c>
+      <c r="D214" t="str">
+        <v>Madhya Pradesh</v>
+      </c>
+      <c r="E214" t="str">
+        <v>Indore (Vijay Nagar)</v>
+      </c>
+      <c r="F214" t="str">
+        <v>Indore Hub</v>
+      </c>
+      <c r="G214" t="str">
+        <v>25 – 34 years (Working Professional / Early Career)</v>
+      </c>
+      <c r="H214" t="str">
+        <v>Female</v>
+      </c>
+      <c r="I214" t="str">
+        <v>Salaried Professional / Corporate Employee</v>
+      </c>
+      <c r="J214" t="str">
+        <v>Rs. 60,001 to Rs. 1,00,000</v>
+      </c>
+      <c r="K214" t="str">
+        <v>3 to 4 times a month</v>
+      </c>
+      <c r="L214" t="str">
+        <v>1 to 2 times a month</v>
+      </c>
+      <c r="M214" t="str">
+        <v>Rs. 1,501 to Rs. 3,000</v>
+      </c>
+      <c r="N214" t="str">
+        <v>Online</v>
+      </c>
+      <c r="O214">
+        <v>4</v>
+      </c>
+      <c r="P214">
+        <v>4</v>
+      </c>
+      <c r="Q214">
+        <v>3</v>
+      </c>
+      <c r="R214">
+        <v>2</v>
+      </c>
+      <c r="S214">
+        <v>5</v>
+      </c>
+      <c r="T214">
+        <v>4</v>
+      </c>
+      <c r="U214">
+        <v>4</v>
+      </c>
+      <c r="V214">
+        <v>5</v>
+      </c>
+      <c r="W214">
+        <v>4</v>
+      </c>
+      <c r="X214" t="str">
+        <v>UPI (Google Pay, PhonePe, Paytm QR)</v>
+      </c>
+      <c r="Y214">
+        <v>5</v>
+      </c>
+      <c r="Z214">
+        <v>4</v>
+      </c>
+      <c r="AA214">
+        <v>4</v>
+      </c>
+      <c r="AB214">
+        <v>4</v>
+      </c>
+      <c r="AC214">
+        <v>3</v>
+      </c>
+      <c r="AD214">
+        <v>5</v>
+      </c>
+      <c r="AE214" t="str">
+        <v>LIVE_RESEARCH_PARTICIPANT</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>RESP-2026-0214</v>
+      </c>
+      <c r="B215" t="str">
+        <v>Dr. Vikramaditya Sharma</v>
+      </c>
+      <c r="C215" t="str">
+        <v>2026-09-20T09:19:28.391Z</v>
+      </c>
+      <c r="D215" t="str">
+        <v>Madhya Pradesh</v>
+      </c>
+      <c r="E215" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="F215" t="str">
+        <v>Indore Hub</v>
+      </c>
+      <c r="G215" t="str">
+        <v>26-35</v>
+      </c>
+      <c r="H215" t="str">
+        <v>Male</v>
+      </c>
+      <c r="I215" t="str">
+        <v>Corporate Professional</v>
+      </c>
+      <c r="J215" t="str">
+        <v>Not Specified</v>
+      </c>
+      <c r="K215" t="str">
+        <v>Frequently (2-3 times a month)</v>
+      </c>
+      <c r="L215" t="str">
+        <v>Occasionally (Once a month)</v>
+      </c>
+      <c r="M215" t="str">
+        <v>₹1,000 - ₹2,500</v>
+      </c>
+      <c r="N215" t="str">
+        <v>Hybrid</v>
+      </c>
+      <c r="O215">
+        <v>4</v>
+      </c>
+      <c r="P215">
+        <v>4</v>
+      </c>
+      <c r="Q215">
+        <v>3</v>
+      </c>
+      <c r="R215">
+        <v>2</v>
+      </c>
+      <c r="S215">
+        <v>5</v>
+      </c>
+      <c r="T215">
+        <v>4</v>
+      </c>
+      <c r="U215">
+        <v>4</v>
+      </c>
+      <c r="V215">
+        <v>5</v>
+      </c>
+      <c r="W215">
+        <v>4</v>
+      </c>
+      <c r="X215" t="str">
+        <v>UPI (Google Pay, PhonePe, Paytm QR)</v>
+      </c>
+      <c r="Y215">
+        <v>5</v>
+      </c>
+      <c r="Z215">
+        <v>4</v>
+      </c>
+      <c r="AA215">
+        <v>3</v>
+      </c>
+      <c r="AB215">
+        <v>4</v>
+      </c>
+      <c r="AC215">
+        <v>2</v>
+      </c>
+      <c r="AD215">
+        <v>5</v>
+      </c>
+      <c r="AE215" t="str">
+        <v>LIVE_RESEARCH_PARTICIPANT</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>RESP-2026-0215</v>
+      </c>
+      <c r="B216" t="str">
+        <v>Priya Sharma (DBA Test)</v>
+      </c>
+      <c r="C216" t="str">
+        <v>2026-09-20T12:42:49.407Z</v>
+      </c>
+      <c r="D216" t="str">
+        <v>Madhya Pradesh</v>
+      </c>
+      <c r="E216" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="F216" t="str">
+        <v>Indore Hub</v>
+      </c>
+      <c r="G216" t="str">
+        <v>26-35</v>
+      </c>
+      <c r="H216" t="str">
+        <v>Female</v>
+      </c>
+      <c r="I216" t="str">
+        <v>Data Architect</v>
+      </c>
+      <c r="J216" t="str">
+        <v>Not Specified</v>
+      </c>
+      <c r="K216" t="str">
+        <v>Frequently (2-3 times a month)</v>
+      </c>
+      <c r="L216" t="str">
+        <v>Occasionally (Once a month)</v>
+      </c>
+      <c r="M216" t="str">
+        <v>₹1,000 - ₹2,500</v>
+      </c>
+      <c r="N216" t="str">
+        <v>Hybrid</v>
+      </c>
+      <c r="O216">
+        <v>4</v>
+      </c>
+      <c r="P216">
+        <v>4</v>
+      </c>
+      <c r="Q216">
+        <v>3</v>
+      </c>
+      <c r="R216">
+        <v>2</v>
+      </c>
+      <c r="S216">
+        <v>5</v>
+      </c>
+      <c r="T216">
+        <v>4</v>
+      </c>
+      <c r="U216">
+        <v>4</v>
+      </c>
+      <c r="V216">
+        <v>5</v>
+      </c>
+      <c r="W216">
+        <v>4</v>
+      </c>
+      <c r="X216" t="str">
+        <v>UPI (Google Pay, PhonePe, Paytm QR)</v>
+      </c>
+      <c r="Y216">
+        <v>5</v>
+      </c>
+      <c r="Z216">
+        <v>4</v>
+      </c>
+      <c r="AA216">
+        <v>3</v>
+      </c>
+      <c r="AB216">
+        <v>4</v>
+      </c>
+      <c r="AC216">
+        <v>2</v>
+      </c>
+      <c r="AD216">
+        <v>5</v>
+      </c>
+      <c r="AE216" t="str">
+        <v>LIVE_RESEARCH_PARTICIPANT</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AE213"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE216"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>